<commit_message>
docs: update death-section rule, runtime checks and release package
</commit_message>
<xml_diff>
--- a/delivery/documents/LDMT_JUNTOS_Final.xlsx
+++ b/delivery/documents/LDMT_JUNTOS_Final.xlsx
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>MVP Final 1</t>
+          <t>MVP Final 2</t>
         </is>
       </c>
       <c r="G6" s="1"/>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>Plataformas de descanso atravessaveis de baixo para cima; inimigo provoca recuperacao conservando estoque/torre.</t>
+          <t>Plataformas de descanso atravessaveis de baixo para cima; morte devolve ao checkpoint e remove blocos construidos de ambos somente na secao atual.</t>
         </is>
       </c>
       <c r="L11" s="11" t="str">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>Recuperacao apos queda maior que 160 px; camera acompanha o jogador mais baixo.</t>
+          <t>Queda maior que 160 px limpa a secao do checkpoint, preserva estoque sem reembolso e mantem plataformas fixas/outras secoes; teste por IDs passou.</t>
         </is>
       </c>
       <c r="L12" s="11" t="str">

</xml_diff>